<commit_message>
Redact customer-specific data from prompts spreadsheet
Replace company name, people, financial figures, quantities,
SKU codes, and TPID with generic placeholders.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Prompts and Responses.xlsx
+++ b/Prompts and Responses.xlsx
@@ -478,7 +478,7 @@
     <row r="2" ht="120" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>When is American Airlines scheduled to sign the MCA-E MACC early renewal?</t>
+          <t>When is Contoso Airlines scheduled to sign the MCA-E MACC early renewal?</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -488,24 +488,24 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
     <row r="3" ht="120" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>What is the TPID and opportunity name for the American Airlines early renewal?</t>
+          <t>What is the TPID and opportunity name for the Contoso Airlines early renewal?</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>TPID is 64422. The opportunity is 'Opportunity Lite: MACC - Azure - Dynamics 365' targeting an MCA-E Early Renewal MACC signature on June 30, 2026.</t>
+          <t>TPID is 12345. The opportunity is 'Opportunity Lite: MACC - Azure - Dynamics 365' targeting an MCA-E Early Renewal MACC signature on June 30, 2026.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
@@ -602,12 +602,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>T-10 (week of Apr 20 – Apr 26). Landing zone readiness for the new region(s) must be confirmed (Kevin), identity/network/security baselines validated, a Day-1 billable workload list created, and migration sequencing aligned to regional availability. Exit: start date options are grounded and feasible.</t>
+          <t>T-10 (week of Apr 20 – Apr 26). Landing zone readiness for the new region(s) must be confirmed (Drew), identity/network/security baselines validated, a Day-1 billable workload list created, and migration sequencing aligned to regional availability. Exit: start date options are grounded and feasible.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
@@ -619,19 +619,19 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>In T-9 (Apr 27 – May 3) Taylor owns the consumption plan v1 workbook and the draft milestone mapping. Named initiatives are populated by Taylor and Abdullah (funding pending flagged). Prabhjot, Farah, and Kevin identify the top 3 growth signals and big bets.</t>
+          <t>In T-9 (Apr 27 – May 3) Jordan owns the consumption plan v1 workbook and the draft milestone mapping. Named initiatives are populated by Jordan and Morgan (funding pending flagged). Casey, Riley, and Drew identify the top 3 growth signals and big bets.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>What current-week activities are in-flight for American Airlines early renewal?</t>
+          <t>What current-week activities are in-flight for Contoso Airlines early renewal?</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx</t>
+          <t>CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>What is Microsoft recommending American Airlines do with Power Apps Premium?</t>
+          <t>What is Microsoft recommending Contoso Airlines do with Power Apps Premium?</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Microsoft recommends that American Airlines standardize on Power Apps Premium for 100% of the Information Worker population at the upcoming Enterprise Agreement milestone — inclusive of approximately 138,000 F SKU frontline employees — with Managed Environments as the default governance posture from day one.</t>
+          <t>Microsoft recommends that Contoso Airlines standardize on Power Apps Premium for 100% of the Information Worker population at the upcoming Enterprise Agreement milestone — inclusive of approximately XXX,XXX F SKU frontline employees — with Managed Environments as the default governance posture from day one.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -665,12 +665,12 @@
     <row r="13" ht="120" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>How many frontline F SKU workers does American Airlines have, and why are they a focus?</t>
+          <t>How many frontline F SKU workers does Contoso Airlines have, and why are they a focus?</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Approximately 138,000 F SKU workers — gate agents, ramp crews, flight attendants, mechanics, cargo handlers, and reservations staff. They are the largest and most operationally impactful cohort at American (multiplying across 6,000+ daily flights) but today run on M365 F3 Basic Power Apps rights only — no premium connectors, no Dataverse, no Managed Environments, no Copilot.</t>
+          <t>Approximately XXX,XXX F SKU workers — gate agents, ramp crews, flight attendants, mechanics, cargo handlers, and reservations staff. They are the largest and most operationally impactful cohort at Contoso (multiplying across 6,000+ daily flights) but today run on M365 F3 Basic Power Apps rights only — no premium connectors, no Dataverse, no Managed Environments, no Copilot.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -716,12 +716,12 @@
     <row r="16" ht="120" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>What four commercial levers are proposed for the 138,000-seat frontline package?</t>
+          <t>What four commercial levers are proposed for the XXX,XXX-seat frontline package?</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>(1) Frontline-Tier Price Point — a Premium add-on to M365 F3 aligned with ratios used for Teams Premium, F-SKU Copilot, and Windows 365 Frontline. (2) Volume-Tier Discounting at 138,000 units qualifying American for top-tier Power Platform volume discount. (3) Coverage Plan Model — Premium for makers/IWs plus a coverage layer for the broader frontline. (4) Displacement Credits from retiring the legacy automation platform and SaaS point-solutions.</t>
+          <t>(1) Frontline-Tier Price Point — a Premium add-on to M365 F3 aligned with ratios used for Teams Premium, F-SKU Copilot, and Windows 365 Frontline. (2) Volume-Tier Discounting at XXX,XXX units qualifying Contoso for top-tier Power Platform volume discount. (3) Coverage Plan Model — Premium for makers/IWs plus a coverage layer for the broader frontline. (4) Displacement Credits from retiring the legacy automation platform and SaaS point-solutions.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Retirement of 100 to 250 legacy applications in the first year through Power Apps modernization, each running on already-owned Premium licenses — turning the investment into an amortizing platform bet rather than a per-project cost center.</t>
+          <t>Retirement of XXX to XXX legacy applications in the first year through Power Apps modernization, each running on already-owned Premium licenses — turning the investment into an amortizing platform bet rather than a per-project cost center.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>1) Standardize Power Apps Premium for 100% of IWs with Managed Environments as default. 2) Structure a 138,000-seat Frontline Premium package using the Coverage Plan model, top-tier volume discounting, and displacement credits. 3) Activate Managed Environments across all production environments within 90 days (Environment Routing, Environment Groups, Solution Checker). 4) Stand up a Power Platform and Copilot CoE co-invested by Microsoft. 5) Launch an Application Modernization Program targeting 100–250 retirements in year one. 6) Commit a first wave of flagship apps (crew reassignment/IRROPS, ramp safety inspection, maintenance triage agent, commercial sales ops, 2–3 mainframe-fronted consoles).</t>
+          <t>1) Standardize Power Apps Premium for 100% of IWs with Managed Environments as default. 2) Structure a XXX,XXX-seat Frontline Premium package using the Coverage Plan model, top-tier volume discounting, and displacement credits. 3) Activate Managed Environments across all production environments within 90 days (Environment Routing, Environment Groups, Solution Checker). 4) Stand up a Power Platform and Copilot CoE co-invested by Microsoft. 5) Launch an Application Modernization Program targeting 100–250 retirements in year one. 6) Commit a first wave of flagship apps (crew reassignment/IRROPS, ramp safety inspection, maintenance triage agent, commercial sales ops, 2–3 mainframe-fronted consoles).</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -784,34 +784,34 @@
     <row r="20" ht="120" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>What is American Airlines' negotiated price for D365 Sales and the ROM to migrate off Siebel SalesLink?</t>
+          <t>What is Contoso Airlines' negotiated price for D365 Sales and the ROM to migrate off Siebel SalesLink?</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>American's negotiated D365 Sales price is $45.98 per user/month. The ROM to migrate SalesLink off Siebel to Dynamics is approximately 2 EDEs, ~1,600 hours at a conservative $400/hour rate, totaling about $700K — with partner options likely lower.</t>
+          <t>Contoso's negotiated D365 Sales price is $XX.XX per user/month. The ROM to migrate SalesLink off Siebel to Dynamics is approximately X EDEs, ~X,XXX hours at a conservative $XXX/hour rate, totaling about $XXXM — with partner options likely lower.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Matthew Bell Estimates for D365 Sales.pdf</t>
+          <t>Alex Johnson Estimates for D365 Sales.pdf</t>
         </is>
       </c>
     </row>
     <row r="21" ht="120" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>What annual incremental Microsoft spend did Matthew Bell estimate if American moves SalesLink to Dynamics?</t>
+          <t>What annual incremental Microsoft spend did Alex Johnson estimate if Contoso moves SalesLink to Dynamics?</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Total up to $574K per year: D365 internal licenses $180K; D365 external users (data packs) $158K; D365 cloud storage incremental $36K; other service-module licenses $200K; Dynamics Portal $10K; Power BI $20K; Azure Function App $20K; Azure OpenAI $150K. American also expects ECIF investment from Microsoft to fund the one-time implementation.</t>
+          <t>Total up to $XXXK per year: D365 internal licenses $XXXK; D365 external users (data packs) $XXXK; D365 cloud storage incremental $XXK; other service-module licenses $XXXK; Dynamics Portal $XXK; Power BI $XXXM; Azure Function App $XXXM; Azure OpenAI $XXXM. Contoso also expects ECIF investment from Microsoft to fund the one-time implementation.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Matthew Bell Estimates for D365 Sales.pdf</t>
+          <t>Alex Johnson Estimates for D365 Sales.pdf</t>
         </is>
       </c>
     </row>
@@ -823,29 +823,29 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Tiered per-100-user packs: $176 per 100-pack up to 9,000 users (e.g., 1,000 users = $1,760/mo; 9,000 = $15,840/mo); $66 per 100-pack from 10,000 to 90,000 users (50,000 = $33,000/mo); $44 per 100-pack at 100,000+ (1,000,000 = $440,000/mo).</t>
+          <t>Tiered per-100-user packs: $XXX per 100-pack up to X,XXX users (e.g., 1,000 users = $X,XXX/mo; X,XXX = $XX,XXX/mo); $XX per 100-pack from XX,XXX to XX,XXX users (XX,XXX = $XX,XXX/mo); $XX per 100-pack at 100,000+ (1,000,000 = $XX0,000/mo).</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Matthew Bell Estimates for D365 Sales.pdf</t>
+          <t>Alex Johnson Estimates for D365 Sales.pdf</t>
         </is>
       </c>
     </row>
     <row r="23" ht="120" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>What attendee structure did Cory Theobald recommend for the BVA discovery calls?</t>
+          <t>What attendee structure did Sam Rivera recommend for the BVA discovery calls?</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>One person from leadership and one from the working team in each functional business unit within scope, with ~45 minutes per call — or one hour if grouping multiple business units. American proposed 9–10am CT Friday, Jan 30 with Pritish Pratap, Minh Duong, Arbind Jaiswal, Rachel Pang, and Matthew Bell.</t>
+          <t>One person from leadership and one from the working team in each functional business unit within scope, with ~45 minutes per call — or one hour if grouping multiple business units. Contoso proposed 9–10am CT Friday, Jan 30 with Pritish Pratap, Minh Duong, Arbind Jaiswal, Rachel Pang, and Alex Johnson.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Matthew Bell Estimates for D365 Sales.pdf</t>
+          <t>Alex Johnson Estimates for D365 Sales.pdf</t>
         </is>
       </c>
     </row>
@@ -857,12 +857,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Year 1 $33.80M; Year 2 $36.74M; Year 3 $38.41M; Year 4 $40.72M; Year 5 $44.09M. Total 5-year EA-Lead spend: approximately $193.77M.</t>
+          <t>Year 1 $XX.XXM; Year 2 $XX.XXM; Year 3 $XX.XXM; Year 4 $XX.XXM; Year 5 $XX.XXM. Total 5-year EA-Lead spend: approximately $XXX.XXM.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model - EXTERNAL.xlsx</t>
+          <t>Contoso Airlines Cost Model - EXTERNAL.xlsx</t>
         </is>
       </c>
     </row>
@@ -874,29 +874,29 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Year 1 As-Is (Illustrative only) EA-Lead annual total is approximately $37.80M, held flat across Years 1–3 for a 3-year total of roughly $113.41M.</t>
+          <t>Year 1 As-Is (Illustrative only) EA-Lead annual total is approximately $XX.XXM, held flat across Years 1–3 for a 3-year total of roughly $XXX.XXM.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model - EXTERNAL.xlsx</t>
+          <t>Contoso Airlines Cost Model - EXTERNAL.xlsx</t>
         </is>
       </c>
     </row>
     <row r="26" ht="120" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>What is the current expiring EA annual run-rate for American Airlines?</t>
+          <t>What is the current expiring EA annual run-rate for Contoso Airlines?</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Expiring Lead annual is about $32.27M, plus Expiring Test of approximately $29.4K — total current expiring annual run-rate of approximately $32.30M.</t>
+          <t>Expiring Lead annual is about $XX.XXM, plus Expiring Test of approximately $XX.XK — total current expiring annual run-rate of approximately $XX.XXM.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model.xlsx</t>
+          <t>Contoso Airlines Cost Model.xlsx</t>
         </is>
       </c>
     </row>
@@ -908,29 +908,29 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>For AAD-33168 (M365 E5 Unified Existing Customer Sub): Year 1 50% discount, Year 2 45%, Year 3 40%, Year 4 35%, Year 5 30% — against a $57 list PUPM. The FSA Renewal SKU (AAD-33177) follows the same discount curve against a $52.11 list.</t>
+          <t>For SKU-XXXXX (M365 E5 Unified Existing Customer Sub): Year 1 XX% discount, Year 2 XX%, Year 3 XX%, Year 4 XX%, Year 5 XX% — against a $XX list PUPM. The FSA Renewal SKU (SKU-XXXXX) follows the same discount curve against a $52.11 list.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model.xlsx</t>
+          <t>Contoso Airlines Cost Model.xlsx</t>
         </is>
       </c>
     </row>
     <row r="28" ht="120" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>What Power Apps Premium quantity is currently on the EA at American Airlines?</t>
+          <t>What Power Apps Premium quantity is currently on the EA at Contoso Airlines?</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>License Details show 19,000 units of Power Apps Premium Sub Per User (20) (SEJ-00016) as a Basic Enterprise Commitment line effective 2026-02-01.</t>
+          <t>License Details show XX,XXX units of Power Apps Premium Sub Per User (20) (SKU-XXXXX) as a Basic Enterprise Commitment line effective 2026-02-01.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model.xlsx</t>
+          <t>Contoso Airlines Cost Model.xlsx</t>
         </is>
       </c>
     </row>
@@ -942,12 +942,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>D365 Sales Sub Per User (DGP-00003): 250 units. D365 Customer Service Sub Per User (DDW-00003): 400 units. D365 Customer Service Attach (SCC-00001): 1,025 units. All Basic Enterprise Commitment lines effective 2026-02-01.</t>
+          <t>D365 Sales Sub Per User (SKU-XXXXX): XXX units. D365 Customer Service Sub Per User (SKU-XXXXX): XXX units. D365 Customer Service Attach (SKU-XXXXX): X,XXX units. All Basic Enterprise Commitment lines effective 2026-02-01.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model.xlsx</t>
+          <t>Contoso Airlines Cost Model.xlsx</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>In-Year Investment layers include: M365 E5 Unified SU (AAD-33196) 32,353 seats at $10.71 PUPM, $4.16M annual; Intune Suite (XQJ-00001) 32,353 seats at 100% discount; M365 Copilot (83I-00001) 10,000 seats at $12 PUPM, $1.44M annual; and Purview Suite FLW (8RL-00005) 134,931 seats at $0.49 PUPM, $788K annual. Total incremental annual ~$6.39M with a 9-month in-year figure around $4.79M.</t>
+          <t>In-Year Investment layers include: M365 E5 Unified SU (SKU-XXXXX) XX,XXX seats at $XX.XX PUPM, $X.XXM annual; Intune Suite (SKU-XXXXX) XX,XXX seats at XX% discount; M365 Copilot (SKU-XXXXX) XX,XXX seats at $12 PUPM, $XX.XXM annual; and Purview Suite FLW (8RL-00005) 134,931 seats at $0.49 PUPM, $XXXM annual. Total incremental annual ~$XX.XXM with a 9-month in-year figure around $XX.XXM.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model - EXTERNAL.xlsx</t>
+          <t>Contoso Airlines Cost Model - EXTERNAL.xlsx</t>
         </is>
       </c>
     </row>
@@ -976,12 +976,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>In American Airlines Cost Model.xlsx the EA-Lead 5-year scenario totals approximately $182.9M across Year 1 $34.42M, Year 2 $35.50M, Year 3 $36.58M, Year 4 $37.66M, and Year 5 $38.74M. The Baseline (expiring-EA flat) comparison totals about $180.71M over the same period.</t>
+          <t>In Contoso Airlines Cost Model.xlsx the EA-Lead 5-year scenario totals approximately $XXX.XM across Year 1 $XX.XXM, Year 2 $XX.XXM, Year 3 $XX.XXM, Year 4 $XX.XXM, and Year 5 $XX.XXM. The Baseline (expiring-EA flat) comparison totals about $XX.XXM over the same period.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model.xlsx</t>
+          <t>Contoso Airlines Cost Model.xlsx</t>
         </is>
       </c>
     </row>
@@ -993,29 +993,29 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>The Early Renewal McCartan workbook mirrors the structure of the standard renewal cost model (summary, M365 E5, Baseline, License Details, PLD, etc.) and is used to reflect the early-renewal sign date of Jun 30, 2026 captured in the walk-back plan. Use it together with the walk-back plan milestones when reviewing pricing, discount curves, and consumption commitments.</t>
+          <t>The Early Renewal Example workbook mirrors the structure of the standard renewal cost model (summary, M365 E5, Baseline, License Details, PLD, etc.) and is used to reflect the early-renewal sign date of Jun 30, 2026 captured in the walk-back plan. Use it together with the walk-back plan milestones when reviewing pricing, discount curves, and consumption commitments.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>American Airlines Cost Model Early Renewal McCartan.xlsx; AA Azure Walk Back Plan.docx</t>
+          <t>Contoso Airlines Cost Model Early Renewal Example.xlsx; CA Azure Walk Back Plan.docx</t>
         </is>
       </c>
     </row>
     <row r="33" ht="120" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Summarize the American Airlines FY26 early renewal in one paragraph.</t>
+          <t>Summarize the Contoso Airlines FY26 early renewal in one paragraph.</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>American Airlines (TPID 64422) is pursuing an early MCA-E MACC renewal targeting a June 30, 2026 signature, with a 12-week walk-back plan from technical readiness (T-10/T-11 in mid-to-late April) through consumption-plan lock (T-8), exec approval (T-6), commercial lock (T-5), final proposal (T-2), and signature readiness (T-1). The commercial envelope is modeled at roughly $183M over five years for the M365 E5 + Defender &amp; Purview FLW + Copilot scenario, with an incremental Power Apps Premium wall-to-wall recommendation covering ~138,000 F-SKU frontline workers and a separate D365 Sales Hub migration track estimated at up to $574K/yr incremental spend plus ~$700K one-time implementation.</t>
+          <t>Contoso Airlines (TPID 12345) is pursuing an early MCA-E MACC renewal targeting a June 30, 2026 signature, with a 12-week walk-back plan from technical readiness (T-10/T-11 in mid-to-late April) through consumption-plan lock (T-8), exec approval (T-6), commercial lock (T-5), final proposal (T-2), and signature readiness (T-1). The commercial envelope is modeled at roughly $XXXM over five years for the M365 E5 + Defender &amp; Purview FLW + Copilot scenario, with an incremental Power Apps Premium wall-to-wall recommendation covering ~XXX,XXX F-SKU frontline workers and a separate D365 Sales Hub migration track estimated at up to $XXXK/yr incremental spend plus ~$XXXM one-time implementation.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx; AA_PowerApps_Premium_Business_Case.docx; American Airlines Cost Model.xlsx; Matthew Bell Estimates for D365 Sales.pdf</t>
+          <t>CA Azure Walk Back Plan.docx; AA_PowerApps_Premium_Business_Case.docx; Contoso Airlines Cost Model.xlsx; Alex Johnson Estimates for D365 Sales.pdf</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Seven files: AA Azure Walk Back Plan.docx (12-week signature plan); AA_PowerApps_Premium_Business_Case.docx (wall-to-wall Power Apps Premium recommendation); AI BP SSP American_Airlines_Early_Renewal_Workback_Plan.docx (MIP-protected, not readable with current permissions); American Airlines Cost Model - EXTERNAL.xlsx (customer-shareable pricing model); American Airlines Cost Model Early Renewal McCartan.xlsx (internal early-renewal working model); American Airlines Cost Model.xlsx (internal renewal model); and Matthew Bell Estimates for D365 Sales.pdf (email thread with D365 Sales Hub budgetary estimates).</t>
+          <t>Seven files: CA Azure Walk Back Plan.docx (12-week signature plan); AA_PowerApps_Premium_Business_Case.docx (wall-to-wall Power Apps Premium recommendation); AI BP SSP Contoso_Airlines_Early_Renewal_Workback_Plan.docx (MIP-protected, not readable with current permissions); Contoso Airlines Cost Model - EXTERNAL.xlsx (customer-shareable pricing model); Contoso Airlines Cost Model Early Renewal Example.xlsx (internal early-renewal working model); Contoso Airlines Cost Model.xlsx (internal renewal model); and Alex Johnson Estimates for D365 Sales.pdf (email thread with D365 Sales Hub budgetary estimates).</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>AA Azure Walk Back Plan.docx; AA_PowerApps_Premium_Business_Case.docx; AI BP SSP American_Airlines_Early_Renewal_Workback_Plan.docx; American Airlines Cost Model - EXTERNAL.xlsx; American Airlines Cost Model Early Renewal McCartan.xlsx; American Airlines Cost Model.xlsx; Matthew Bell Estimates for D365 Sales.pdf</t>
+          <t>CA Azure Walk Back Plan.docx; AA_PowerApps_Premium_Business_Case.docx; AI BP SSP Contoso_Airlines_Early_Renewal_Workback_Plan.docx; Contoso Airlines Cost Model - EXTERNAL.xlsx; Contoso Airlines Cost Model Early Renewal Example.xlsx; Contoso Airlines Cost Model.xlsx; Alex Johnson Estimates for D365 Sales.pdf</t>
         </is>
       </c>
     </row>
@@ -1040,10 +1040,4 @@
   <autoFilter ref="A1:C34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{f42aa342-8706-4288-bd11-ebb85995028c}" enabled="1" method="Privileged" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" removed="0"/>
-</clbl:labelList>
 </file>
</xml_diff>